<commit_message>
Englisch: „Invoice (bank transfer)“ statt „Bank transfer by invoice“, „room history“ einheitlich (Hinweise des Gegenlesers geprüft)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sessions/Uebersetzung-en-neu-seit-Gegenlesen.xlsx
+++ b/Sessions/Uebersetzung-en-neu-seit-Gegenlesen.xlsx
@@ -241,8 +241,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Texte_help" displayName="Texte_help" ref="A1:G14" headerRowCount="1">
-  <autoFilter ref="A1:G14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Texte_help" displayName="Texte_help" ref="A1:G15" headerRowCount="1">
+  <autoFilter ref="A1:G15"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Schlüssel"/>
     <tableColumn id="2" name="Ort"/>
@@ -707,7 +707,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>• Hilfe und Lotsen (13 Texte): Leser sind Rezeption, Inhaber und Manager. Erklärend; Namen von Knöpfen und Seiten in Anführungszeichen wortgleich mit der Oberfläche. „Lotse“ heißt „guide“.</t>
+          <t>• Hilfe und Lotsen (14 Texte): Leser sind Rezeption, Inhaber und Manager. Erklärend; Namen von Knöpfen und Seiten in Anführungszeichen wortgleich mit der Oberfläche. „Lotse“ heißt „guide“.</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Zusammen 1236 Texte · erzeugt aus src/lib/i18n/</t>
+          <t>Zusammen 1237 Texte · erzeugt aus src/lib/i18n/</t>
         </is>
       </c>
     </row>
@@ -27638,7 +27638,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Bank transfer by invoice</t>
+          <t>Invoice (bank transfer)</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr"/>
@@ -30277,7 +30277,7 @@
       </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
-          <t>No payment method yet. Three options, all through our payment provider Stripe: card or SEPA direct debit are stored here and collected monthly; with bank transfer by invoice, nothing is stored, and every invoice states bank details with a payment reference.</t>
+          <t>No payment method yet. Three options, all through our payment provider Stripe: card or SEPA direct debit are stored here and collected monthly; with invoice and bank transfer, nothing is stored, and every invoice states bank details with a payment reference.</t>
         </is>
       </c>
       <c r="F95" s="7" t="inlineStr"/>
@@ -30393,7 +30393,7 @@
       </c>
       <c r="E99" s="6" t="inlineStr">
         <is>
-          <t>Bank transfer by invoice</t>
+          <t>Invoice (bank transfer)</t>
         </is>
       </c>
       <c r="F99" s="7" t="inlineStr"/>
@@ -30422,7 +30422,7 @@
       </c>
       <c r="E100" s="6" t="inlineStr">
         <is>
-          <t>Bank transfer by invoice selected.</t>
+          <t>Invoice (bank transfer) selected.</t>
         </is>
       </c>
       <c r="F100" s="7" t="inlineStr"/>
@@ -30741,7 +30741,7 @@
       </c>
       <c r="E111" s="6" t="inlineStr">
         <is>
-          <t>Rather not store a card or account? &lt;link&gt;Choose bank transfer by invoice&lt;/link&gt; — every invoice then states bank details and a payment reference, payment term 14 days.</t>
+          <t>Rather not store a card or account? &lt;link&gt;Choose invoice (bank transfer)&lt;/link&gt; — every invoice then states bank details and a payment reference, payment term 14 days.</t>
         </is>
       </c>
       <c r="F111" s="7" t="inlineStr"/>
@@ -30857,7 +30857,7 @@
       </c>
       <c r="E115" s="6" t="inlineStr">
         <is>
-          <t>Bank transfer by invoice</t>
+          <t>Invoice (bank transfer)</t>
         </is>
       </c>
       <c r="F115" s="7" t="inlineStr"/>
@@ -36363,7 +36363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -36464,7 +36464,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>In the room’s history, the “Check-out” entry links to the statement. This is not an invoice: it contains no guest name, invoice number, or tax breakdown. It shows the amount to be collected.</t>
+          <t>In the room history, the “Check-out” entry links to the statement. This is not an invoice: it contains no guest name, invoice number, or tax breakdown. It shows the amount to be collected.</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr"/>
@@ -36493,7 +36493,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Cleaning becomes available at that time. Either the guest selected “not before” in the portal or asked the housekeeper at the door to come back later. The room’s history shows which. Until then, the room isn’t available for cleaning on either board; it opens automatically at the specified time. How long guests may postpone in the portal is set under Property &amp; rules.</t>
+          <t>Cleaning becomes available at that time. Either the guest selected “not before” in the portal or asked the housekeeper at the door to come back later. The room history shows which. Until then, the room isn’t available for cleaning on either board; it opens automatically at the specified time. How long guests may postpone in the portal is set under Property &amp; rules.</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr"/>
@@ -36522,7 +36522,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>The 20 most recent requests appear collapsed below the open requests. Beyond that, every request remains available in the room’s history for 30 days and, if it carried a price, on the stay statement.</t>
+          <t>The 20 most recent requests appear collapsed below the open requests. Beyond that, every request remains available in the room history for 30 days and, if it carried a price, on the stay statement.</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr"/>
@@ -36531,7 +36531,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>topics.zimmer.bloecke.1.eintraege.3.antwort</t>
+          <t>topics.anfragen.bloecke.2.eintraege.5.antwort</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -36546,12 +36546,12 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Außer Betrieb ist der empfohlene Weg für Renovierung und Stilllegung: kein Check-in, nicht auf dem Reinigungsboard, nicht auf den Aushängen – aber alles bleibt erhalten, und ein Klick holt das Zimmer zurück. Die Nummer bleibt dabei belegt. Löschen ist endgültig und gibt die Nummer frei.</t>
+          <t>Prüfen Sie im Verlauf des Zimmers, ob eine Anfrage angekommen ist. Häufigste Ursachen: Der Gast hat vor dem Absenden abgebrochen, oder er hat eine Kachel unter „Nützliche Links“ benutzt, etwa einen Lieferdienst – die führt nach außen und erzeugt keine Anfrage.</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>For renovations or temporary closures, we recommend marking the room “Out of service”: it can’t be checked into, doesn’t appear on the housekeeping board or room signs, and all its history is retained. One click restores it to service, and the room number remains reserved. Deleting a room is permanent and frees the room number.</t>
+          <t>Check the room history to see whether a request arrived. The most common causes: the guest canceled before sending, or used a tile under “Useful links,” such as a food delivery service — that leads to an outside site and doesn’t create a request.</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr"/>
@@ -36560,7 +36560,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>topics.gastzugang.bloecke.1.eintraege.0.antwort</t>
+          <t>topics.zimmer.bloecke.1.eintraege.3.antwort</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -36575,12 +36575,12 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Fester QR + PIN, wenn Sie in den Zimmern einen Aushang aufstellen oder anbringen können und zwei Faktoren wollen (Code im Zimmer, PIN vom Tresen). Individueller Zugang, wenn Aushänge nicht möglich oder nicht gewünscht sind – bequemer für den Gast, aber wer das Blatt sieht, hat Zugang. Die Seite stellt beides ausführlich gegenüber.</t>
+          <t>Außer Betrieb ist der empfohlene Weg für Renovierung und Stilllegung: kein Check-in, nicht auf dem Reinigungsboard, nicht auf den Aushängen – aber alles bleibt erhalten, und ein Klick holt das Zimmer zurück. Die Nummer bleibt dabei belegt. Löschen ist endgültig und gibt die Nummer frei.</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Choose fixed QR code + PIN if you can display a sign in each room and want two-factor access (the code in the room and the PIN from the front desk). Choose personal access if signs aren’t practical or desired. It’s more convenient for guests, but anyone who sees the sheet can access the portal for that stay. The page compares both in detail.</t>
+          <t>For renovations or temporary closures, we recommend marking the room “Out of service”: it can’t be checked into, doesn’t appear on the housekeeping board or room signs, and all its history is retained. One click restores it to service, and the room number remains reserved. Deleting a room is permanent and frees the room number.</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr"/>
@@ -36589,7 +36589,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>topics.services.bloecke.2.eintraege.6.antwort</t>
+          <t>topics.gastzugang.bloecke.1.eintraege.0.antwort</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -36604,12 +36604,12 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Eine Kachel im Gästeportal, die einen Link nach außen öffnet – etwa die Trinkgeld-App fürs Reinigungsteam, ein Lieferdienst oder ein Taxi. Ein Verweis erzeugt keine Anfrage: nichts auf dem Board, nichts auf der Aufstellung. Vorlagen füllen das Formular vor; die Adresse passen Sie auf Ihr Konto oder Ihre Stadt an. Das Portal bettet nichts ein, es verlinkt nur – für das Ziel ist der Anbieter verantwortlich.</t>
+          <t>Fester QR + PIN, wenn Sie in den Zimmern einen Aushang aufstellen oder anbringen können und zwei Faktoren wollen (Code im Zimmer, PIN vom Tresen). Individueller Zugang, wenn Aushänge nicht möglich oder nicht gewünscht sind – bequemer für den Gast, aber wer das Blatt sieht, hat Zugang. Die Seite stellt beides ausführlich gegenüber.</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>A tile in the guest portal that links to an external website, such as a tipping app for the housekeeping team, a food delivery service, or a taxi service. A link doesn’t create a request, so nothing appears on the Requests page or the stay statement. Templates prefill the form; adjust the address to your account or city. The portal only links to the external service; the provider is responsible for its content.</t>
+          <t>Choose fixed QR code + PIN if you can display a sign in each room and want two-factor access (the code in the room and the PIN from the front desk). Choose personal access if signs aren’t practical or desired. It’s more convenient for guests, but anyone who sees the sheet can access the portal for that stay. The page compares both in detail.</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr"/>
@@ -36618,7 +36618,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>topics.auswertung.bloecke.0.absaetze.0</t>
+          <t>topics.services.bloecke.2.eintraege.6.antwort</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -36633,12 +36633,12 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Alles hier ist gerechnet, nichts gespeichert: Grundlage sind die Einträge der Reinigungskräfte (Schichtbeginn und -ende, Pause, sonstige Reinigung, Start und Abschluss je Zimmer) sowie Gast-Tipps und Check-outs. Der Zeitraum steht in der Adresse – ein Stand lässt sich verlinken und drucken.</t>
+          <t>Eine Kachel im Gästeportal, die einen Link nach außen öffnet – etwa die Trinkgeld-App fürs Reinigungsteam, ein Lieferdienst oder ein Taxi. Ein Verweis erzeugt keine Anfrage: nichts auf dem Board, nichts auf der Aufstellung. Vorlagen füllen das Formular vor; die Adresse passen Sie auf Ihr Konto oder Ihre Stadt an. Das Portal bettet nichts ein, es verlinkt nur – für das Ziel ist der Anbieter verantwortlich.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Everything here is calculated, not stored. It’s based on housekeepers’ entries (shift start and end, breaks, other cleaning, and start and finish times for each room), plus guest taps and check-outs. The selected period appears in the web address, so you can share or print a snapshot.</t>
+          <t>A tile in the guest portal that links to an external website, such as a tipping app for the housekeeping team, a food delivery service, or a taxi service. A link doesn’t create a request, so nothing appears on the Requests page or the stay statement. Templates prefill the form; adjust the address to your account or city. The portal only links to the external service; the provider is responsible for its content.</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr"/>
@@ -36647,27 +36647,27 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>ui.hub.intro</t>
+          <t>topics.auswertung.bloecke.0.absaetze.0</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Bedienelemente der Hilfe: „?“-Knopf, Leiste, Lotsen-Karte, Hilfe-Hub</t>
+          <t>Hilfe-Leiste neben der Seite bzw. Hilfe-Themenseite</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Kurz. {title} = Thema, {step}/{total} = Schritt, {done}/{total} = erledigte Punkte, {count} = Schritte.</t>
+          <t>Titel und Untertitel eines Themas, Absätze, Legenden (Beschriftung eines Zeichens + Erklärung), Fragen mit Antworten, Verweise auf andere Themen. Uhrzeiten im 24-Stunden-Format; Namen von Knöpfen wortgleich mit der Oberfläche.</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Zu jedem Bereich gibt es eine Erklärung zum Nachschlagen – Zeichen, Fragen, Antworten – und einen Lotsen: einen geführten Rundgang über die echte Seite, der Schritt für Schritt zeigt, was dort womit passiert. Bedienen können Sie die Seite dabei ganz normal weiter, nichts ist gesperrt; beenden lässt sich der Lotse jederzeit über „Beenden“. Das „?“ oben rechts klappt auf jeder Seite die Erklärung daneben auf.</t>
+          <t>Alles hier ist gerechnet, nichts gespeichert: Grundlage sind die Einträge der Reinigungskräfte (Schichtbeginn und -ende, Pause, sonstige Reinigung, Start und Abschluss je Zimmer) sowie Gast-Tipps und Check-outs. Der Zeitraum steht in der Adresse – ein Stand lässt sich verlinken und drucken.</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Each area has an explanation to look things up — symbols, questions, and answers — plus a guide: a guided tour of the actual page that shows you step by step how it works. You can continue using the page normally; nothing is locked. End the guide at any time with “End.” The “?” in the top-right corner opens the explanation beside any page.</t>
+          <t>Everything here is calculated, not stored. It’s based on housekeepers’ entries (shift start and end, breaks, other cleaning, and start and finish times for each room), plus guest taps and check-outs. The selected period appears in the web address, so you can share or print a snapshot.</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr"/>
@@ -36676,7 +36676,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>ui.hub.catalogIntro</t>
+          <t>ui.hub.intro</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -36691,12 +36691,12 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Beides führt auf die Seite, um die es geht: die Erklärung zum Nachschlagen in der Leiste daneben, der Lotse Schritt für Schritt darüber – beliebig oft.</t>
+          <t>Zu jedem Bereich gibt es eine Erklärung zum Nachschlagen – Zeichen, Fragen, Antworten – und einen Lotsen: einen geführten Rundgang über die echte Seite, der Schritt für Schritt zeigt, was dort womit passiert. Bedienen können Sie die Seite dabei ganz normal weiter, nichts ist gesperrt; beenden lässt sich der Lotse jederzeit über „Beenden“. Das „?“ oben rechts klappt auf jeder Seite die Erklärung daneben auf.</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Both take you to the relevant page: the explanation opens in the sidebar, while the guide walks you through the page step by step. You can use either as often as you like.</t>
+          <t>Each area has an explanation to look things up — symbols, questions, and answers — plus a guide: a guided tour of the actual page that shows you step by step how it works. You can continue using the page normally; nothing is locked. End the guide at any time with “End.” The “?” in the top-right corner opens the explanation beside any page.</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr"/>
@@ -36705,27 +36705,27 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>sim.reinigung.page.intro</t>
+          <t>ui.hub.catalogIntro</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Nachbauten von Reinigungsboard und Gästeportal im Hilfe-Bereich</t>
+          <t>Bedienelemente der Hilfe: „?“-Knopf, Leiste, Lotsen-Karte, Hilfe-Hub</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Beispielwerte (Hausname, Services) frei übersetzen; Preise im Format der Sprache. {path} = Adresse, {count} = Anzahl.</t>
+          <t>Kurz. {title} = Thema, {step}/{total} = Schritt, {done}/{total} = erledigte Punkte, {count} = Schritte.</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>So sieht das Board aus, das Ihre Reinigungskräfte am Handy bedienen. Es ist ein Nachbau mit Beispiel-Zimmern – hier wird nichts gespeichert und niemand benachrichtigt. Probieren Sie ruhig alles aus; der Lotse stellt zu jedem Schritt die passende Ansicht wieder her.</t>
+          <t>Beides führt auf die Seite, um die es geht: die Erklärung zum Nachschlagen in der Leiste daneben, der Lotse Schritt für Schritt darüber – beliebig oft.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>This is the board your housekeepers use on their phones. It’s a replica with sample rooms; nothing is saved and no one is notified. Feel free to try everything. The guide restores the appropriate view at each step.</t>
+          <t>Both take you to the relevant page: the explanation opens in the sidebar, while the guide walks you through the page step by step. You can use either as often as you like.</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr"/>
@@ -36734,7 +36734,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>sim.reinigung.page.why</t>
+          <t>sim.reinigung.page.intro</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -36749,12 +36749,12 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Warum ein Nachbau und keine Führung durch das echte Board? Das Reinigungsboard hat eine eigene Anmeldung und eine eigene Sitzung – aus der Rezeption heraus ist es nicht erreichbar. Wer es wirklich sehen will, meldet sich unter &lt;code&gt;{path}&lt;/code&gt; mit dem Zugang einer Reinigungskraft an.</t>
+          <t>So sieht das Board aus, das Ihre Reinigungskräfte am Handy bedienen. Es ist ein Nachbau mit Beispiel-Zimmern – hier wird nichts gespeichert und niemand benachrichtigt. Probieren Sie ruhig alles aus; der Lotse stellt zu jedem Schritt die passende Ansicht wieder her.</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Why a replica instead of a tour of the live board? The housekeeping board has its own sign-in and session, so it can’t be accessed from the front desk. To see the live board, sign in at &lt;code&gt;{path}&lt;/code&gt; using a housekeeper’s account.</t>
+          <t>This is the board your housekeepers use on their phones. It’s a replica with sample rooms; nothing is saved and no one is notified. Feel free to try everything. The guide restores the appropriate view at each step.</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr"/>
@@ -36763,7 +36763,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>sim.gast.page.intro</t>
+          <t>sim.reinigung.page.why</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -36778,16 +36778,45 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Das Gästeportal, wie es auf dem Telefon Ihres Gastes aussieht. Ein Nachbau mit Beispielwerten – Haus, Zimmer und Services stammen nicht aus Ihren Daten, damit die Ansicht auch dann etwas zeigt, wenn noch nichts angelegt ist. Nichts davon wird gespeichert.</t>
+          <t>Warum ein Nachbau und keine Führung durch das echte Board? Das Reinigungsboard hat eine eigene Anmeldung und eine eigene Sitzung – aus der Rezeption heraus ist es nicht erreichbar. Wer es wirklich sehen will, meldet sich unter &lt;code&gt;{path}&lt;/code&gt; mit dem Zugang einer Reinigungskraft an.</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>This is what the guest portal looks like on a guest’s phone. It’s a replica with sample data; the property, room, and services don’t come from your data, so the screen shows something even before setup is complete. Nothing is saved.</t>
+          <t>Why a replica instead of a tour of the live board? The housekeeping board has its own sign-in and session, so it can’t be accessed from the front desk. To see the live board, sign in at &lt;code&gt;{path}&lt;/code&gt; using a housekeeper’s account.</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr"/>
       <c r="G14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>sim.gast.page.intro</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Nachbauten von Reinigungsboard und Gästeportal im Hilfe-Bereich</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Beispielwerte (Hausname, Services) frei übersetzen; Preise im Format der Sprache. {path} = Adresse, {count} = Anzahl.</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Das Gästeportal, wie es auf dem Telefon Ihres Gastes aussieht. Ein Nachbau mit Beispielwerten – Haus, Zimmer und Services stammen nicht aus Ihren Daten, damit die Ansicht auch dann etwas zeigt, wenn noch nichts angelegt ist. Nichts davon wird gespeichert.</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>This is what the guest portal looks like on a guest’s phone. It’s a replica with sample data; the property, room, and services don’t come from your data, so the screen shows something even before setup is complete. Nothing is saved.</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr"/>
+      <c r="G15" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>